<commit_message>
Update seed data to latest HR Excel (96 employees, clean)
Regenerated the default dataset from the newly uploaded Excel through the real
ingestion pipeline. 96 permanent employees, data-quality 100 (0 invalid, 0
duplicates, 0 missing), Saudization 39.6%, kind=permanent active snapshot;
sample updated to match. Verified on a fresh boot with no errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BjKdiq6boxtc7yT3vRmLB6
</commit_message>
<xml_diff>
--- a/data/samples/HR_Current.xlsx
+++ b/data/samples/HR_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DeLL\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C97BA13D-241E-4692-998C-1939EA67AFD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{276C00FB-54C1-44EA-9C14-1FF62F03E87A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5580" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{B35A5613-5B32-42A3-89F3-C94ABABE9032}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="262">
   <si>
     <t>Employee Code</t>
   </si>
@@ -487,6 +487,339 @@
   </si>
   <si>
     <t>عبد العزيز حجيج رضيمان المرواني</t>
+  </si>
+  <si>
+    <t>MD Sahidul Islam</t>
+  </si>
+  <si>
+    <t>مد سيدول اسلام</t>
+  </si>
+  <si>
+    <t>الإشراف الداخلي - فندق ميسان روتانا المسك</t>
+  </si>
+  <si>
+    <t>Houseman</t>
+  </si>
+  <si>
+    <t>المدينة - الحربي</t>
+  </si>
+  <si>
+    <t>Samim Hossain</t>
+  </si>
+  <si>
+    <t>شميم اوسين</t>
+  </si>
+  <si>
+    <t>Md Hamidul Islam</t>
+  </si>
+  <si>
+    <t>مد حميد ال اسلام</t>
+  </si>
+  <si>
+    <t>Md Belal Hossen</t>
+  </si>
+  <si>
+    <t>مد حسين بلال</t>
+  </si>
+  <si>
+    <t>Md Sujib Mia</t>
+  </si>
+  <si>
+    <t>مد سوجيب مياه</t>
+  </si>
+  <si>
+    <t>الإشراف الداخلي - فندق ميسان التقوى</t>
+  </si>
+  <si>
+    <t>Morshed Alam</t>
+  </si>
+  <si>
+    <t>مرشد علام</t>
+  </si>
+  <si>
+    <t>SOHAG MIA</t>
+  </si>
+  <si>
+    <t>شوهاك مد عزيز الحكيم ميا</t>
+  </si>
+  <si>
+    <t>Anowar Hossain</t>
+  </si>
+  <si>
+    <t>انور اوسين</t>
+  </si>
+  <si>
+    <t>Md Rubel Miah</t>
+  </si>
+  <si>
+    <t>مد روبيل مياه</t>
+  </si>
+  <si>
+    <t>حاملي الحقائب - ميسان رحاب المسك</t>
+  </si>
+  <si>
+    <t>حامل حقائب</t>
+  </si>
+  <si>
+    <t>Zakir Hossain</t>
+  </si>
+  <si>
+    <t>زاكير اوسين</t>
+  </si>
+  <si>
+    <t>Md Sahajahan</t>
+  </si>
+  <si>
+    <t>مد شاه جهان</t>
+  </si>
+  <si>
+    <t>Md Jamil Hossen</t>
+  </si>
+  <si>
+    <t>مد جميل حسين</t>
+  </si>
+  <si>
+    <t>Sohel Sayedol Hoque</t>
+  </si>
+  <si>
+    <t>سهيل سعيد هوكي هوكي</t>
+  </si>
+  <si>
+    <t>Muhammad Meer Hossion</t>
+  </si>
+  <si>
+    <t>محمد مير حوسيون</t>
+  </si>
+  <si>
+    <t>Foaiz Ullah</t>
+  </si>
+  <si>
+    <t>فيض الله</t>
+  </si>
+  <si>
+    <t>Md Roman Miah</t>
+  </si>
+  <si>
+    <t>مد رومان مياه</t>
+  </si>
+  <si>
+    <t>Md Rahad</t>
+  </si>
+  <si>
+    <t>مد راهاد راهاد مد</t>
+  </si>
+  <si>
+    <t>MD Shahidul Islam</t>
+  </si>
+  <si>
+    <t>مد شهيد الاسلام</t>
+  </si>
+  <si>
+    <t>المدينة - موارد</t>
+  </si>
+  <si>
+    <t>Estiek Hossain</t>
+  </si>
+  <si>
+    <t>اشتياق حسين</t>
+  </si>
+  <si>
+    <t>MD Somon Miah</t>
+  </si>
+  <si>
+    <t>مد شمون مياه</t>
+  </si>
+  <si>
+    <t>المدينة - جبل احد</t>
+  </si>
+  <si>
+    <t>Mohammed Yeasin Arafat</t>
+  </si>
+  <si>
+    <t>محمد ياسين عرفات</t>
+  </si>
+  <si>
+    <t>Naim Howlader</t>
+  </si>
+  <si>
+    <t>نعيم حولادر</t>
+  </si>
+  <si>
+    <t>Md Alamin Mia</t>
+  </si>
+  <si>
+    <t>محمد لامين ميا</t>
+  </si>
+  <si>
+    <t>MD Mizanur Rahman</t>
+  </si>
+  <si>
+    <t>مد ميزان نور رحمن</t>
+  </si>
+  <si>
+    <t>Rakib Hossain</t>
+  </si>
+  <si>
+    <t>رقيب حسين</t>
+  </si>
+  <si>
+    <t>MD Faruq</t>
+  </si>
+  <si>
+    <t>مد قاروق</t>
+  </si>
+  <si>
+    <t>Ahmadulla Mamun</t>
+  </si>
+  <si>
+    <t>أحمد الله مامون</t>
+  </si>
+  <si>
+    <t>Mohammad Jihad Hossain</t>
+  </si>
+  <si>
+    <t>محمد جهاد حسين</t>
+  </si>
+  <si>
+    <t>Alamin Abo Taher</t>
+  </si>
+  <si>
+    <t>الامين ابو الطاهر</t>
+  </si>
+  <si>
+    <t>MD Nobibur Rahman</t>
+  </si>
+  <si>
+    <t>مد نوبيب ال رحمن</t>
+  </si>
+  <si>
+    <t>MD Joynal Mia</t>
+  </si>
+  <si>
+    <t>مد جونيال ميا</t>
+  </si>
+  <si>
+    <t>MD Ahnaf</t>
+  </si>
+  <si>
+    <t>مد احناف</t>
+  </si>
+  <si>
+    <t>حاملي الحقائب - فندق ميسان روتانا المسك</t>
+  </si>
+  <si>
+    <t>المدينة - ارض النظافة</t>
+  </si>
+  <si>
+    <t>Shahriar Nawas</t>
+  </si>
+  <si>
+    <t>شهريار نواز</t>
+  </si>
+  <si>
+    <t>Sarif Hannan</t>
+  </si>
+  <si>
+    <t>شريف حنان</t>
+  </si>
+  <si>
+    <t>Junaed Md Jamir Ali</t>
+  </si>
+  <si>
+    <t>جوند محمد جامير علي علي</t>
+  </si>
+  <si>
+    <t>Md Shakhawat Hossain</t>
+  </si>
+  <si>
+    <t>مد شخوات اوسين</t>
+  </si>
+  <si>
+    <t>Md Al Amin</t>
+  </si>
+  <si>
+    <t>مد ال أمين</t>
+  </si>
+  <si>
+    <t>Md Shakil Rana</t>
+  </si>
+  <si>
+    <t>مد شكيل رنا</t>
+  </si>
+  <si>
+    <t>Alif Hasan Rabby</t>
+  </si>
+  <si>
+    <t>اليف حسان ربي</t>
+  </si>
+  <si>
+    <t>Md Uzzal Mia</t>
+  </si>
+  <si>
+    <t>مد اوزال ميا</t>
+  </si>
+  <si>
+    <t>Mohammad Abu Tahar</t>
+  </si>
+  <si>
+    <t>محمد ابو طاهر ابو طاهر طاهر</t>
+  </si>
+  <si>
+    <t>Md Jishan</t>
+  </si>
+  <si>
+    <t>مد جيشان</t>
+  </si>
+  <si>
+    <t>Faysal Pathan</t>
+  </si>
+  <si>
+    <t>فيصل باثين كاشم باتهان</t>
+  </si>
+  <si>
+    <t>Mohammad Monir</t>
+  </si>
+  <si>
+    <t>محمد منير</t>
+  </si>
+  <si>
+    <t>MOHAMMAD HUMAYUN</t>
+  </si>
+  <si>
+    <t>محمد هومايون منصور علي</t>
+  </si>
+  <si>
+    <t>Asst. Catering Manager</t>
+  </si>
+  <si>
+    <t>MD Shakayet Turaz</t>
+  </si>
+  <si>
+    <t>مد شاكيت توراز</t>
+  </si>
+  <si>
+    <t>Saif Al Mohamed Islam Islam</t>
+  </si>
+  <si>
+    <t>سيف ال محمد اسلام اسلام</t>
+  </si>
+  <si>
+    <t>AHAMMAD ALI MAFIJ UDDIN</t>
+  </si>
+  <si>
+    <t>احمد علي مفيض دين</t>
+  </si>
+  <si>
+    <t>SAFIULLAH ABDUL KADIR</t>
+  </si>
+  <si>
+    <t>صفي الله عبد ال قادر</t>
+  </si>
+  <si>
+    <t>Sakawat Hossen</t>
+  </si>
+  <si>
+    <t>سخاوات اوسين</t>
   </si>
 </sst>
 </file>
@@ -840,7 +1173,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{883B3F3C-5A92-453D-9638-D2640977E06C}">
-  <dimension ref="A1:T47"/>
+  <dimension ref="A1:T97"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -3262,6 +3595,2704 @@
         <v>25</v>
       </c>
     </row>
+    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>2651</v>
+      </c>
+      <c r="C48" t="s">
+        <v>151</v>
+      </c>
+      <c r="D48" t="s">
+        <v>152</v>
+      </c>
+      <c r="E48">
+        <v>6</v>
+      </c>
+      <c r="F48" t="s">
+        <v>46</v>
+      </c>
+      <c r="G48" t="s">
+        <v>153</v>
+      </c>
+      <c r="H48" t="s">
+        <v>154</v>
+      </c>
+      <c r="I48">
+        <v>2800</v>
+      </c>
+      <c r="J48">
+        <v>0</v>
+      </c>
+      <c r="K48">
+        <v>0</v>
+      </c>
+      <c r="L48" t="s">
+        <v>23</v>
+      </c>
+      <c r="M48" t="s">
+        <v>40</v>
+      </c>
+      <c r="N48" s="1">
+        <v>46244</v>
+      </c>
+      <c r="P48" s="1">
+        <v>46243</v>
+      </c>
+      <c r="R48" s="1">
+        <v>46006</v>
+      </c>
+      <c r="T48" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="49" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49">
+        <v>6126</v>
+      </c>
+      <c r="C49" t="s">
+        <v>156</v>
+      </c>
+      <c r="D49" t="s">
+        <v>157</v>
+      </c>
+      <c r="E49">
+        <v>6</v>
+      </c>
+      <c r="F49" t="s">
+        <v>37</v>
+      </c>
+      <c r="G49" t="s">
+        <v>38</v>
+      </c>
+      <c r="H49" t="s">
+        <v>154</v>
+      </c>
+      <c r="I49">
+        <v>2800</v>
+      </c>
+      <c r="J49">
+        <v>0</v>
+      </c>
+      <c r="K49">
+        <v>0</v>
+      </c>
+      <c r="L49" t="s">
+        <v>23</v>
+      </c>
+      <c r="M49" t="s">
+        <v>40</v>
+      </c>
+      <c r="N49" s="1">
+        <v>45645</v>
+      </c>
+      <c r="O49" s="1">
+        <v>46009</v>
+      </c>
+      <c r="P49" s="1">
+        <v>45734</v>
+      </c>
+      <c r="R49" s="1">
+        <v>45673</v>
+      </c>
+      <c r="T49" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="50" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50">
+        <v>6127</v>
+      </c>
+      <c r="C50" t="s">
+        <v>158</v>
+      </c>
+      <c r="D50" t="s">
+        <v>159</v>
+      </c>
+      <c r="E50">
+        <v>6</v>
+      </c>
+      <c r="F50" t="s">
+        <v>37</v>
+      </c>
+      <c r="G50" t="s">
+        <v>38</v>
+      </c>
+      <c r="H50" t="s">
+        <v>154</v>
+      </c>
+      <c r="I50">
+        <v>2800</v>
+      </c>
+      <c r="J50">
+        <v>0</v>
+      </c>
+      <c r="K50">
+        <v>0</v>
+      </c>
+      <c r="L50" t="s">
+        <v>23</v>
+      </c>
+      <c r="M50" t="s">
+        <v>40</v>
+      </c>
+      <c r="N50" s="1">
+        <v>45645</v>
+      </c>
+      <c r="O50" s="1">
+        <v>46009</v>
+      </c>
+      <c r="P50" s="1">
+        <v>45734</v>
+      </c>
+      <c r="R50" s="1">
+        <v>45006</v>
+      </c>
+      <c r="T50" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <v>6129</v>
+      </c>
+      <c r="C51" t="s">
+        <v>160</v>
+      </c>
+      <c r="D51" t="s">
+        <v>161</v>
+      </c>
+      <c r="E51">
+        <v>6</v>
+      </c>
+      <c r="F51" t="s">
+        <v>37</v>
+      </c>
+      <c r="G51" t="s">
+        <v>38</v>
+      </c>
+      <c r="H51" t="s">
+        <v>154</v>
+      </c>
+      <c r="I51">
+        <v>2800</v>
+      </c>
+      <c r="J51">
+        <v>0</v>
+      </c>
+      <c r="K51">
+        <v>0</v>
+      </c>
+      <c r="L51" t="s">
+        <v>23</v>
+      </c>
+      <c r="M51" t="s">
+        <v>40</v>
+      </c>
+      <c r="N51" s="1">
+        <v>45901</v>
+      </c>
+      <c r="O51" s="1">
+        <v>46265</v>
+      </c>
+      <c r="P51" s="1">
+        <v>45990</v>
+      </c>
+      <c r="R51" s="1">
+        <v>46250</v>
+      </c>
+      <c r="T51" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="52" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52">
+        <v>6145</v>
+      </c>
+      <c r="C52" t="s">
+        <v>162</v>
+      </c>
+      <c r="D52" t="s">
+        <v>163</v>
+      </c>
+      <c r="E52">
+        <v>6</v>
+      </c>
+      <c r="F52" t="s">
+        <v>66</v>
+      </c>
+      <c r="G52" t="s">
+        <v>164</v>
+      </c>
+      <c r="H52" t="s">
+        <v>154</v>
+      </c>
+      <c r="I52">
+        <v>2800</v>
+      </c>
+      <c r="J52">
+        <v>0</v>
+      </c>
+      <c r="K52">
+        <v>0</v>
+      </c>
+      <c r="L52" t="s">
+        <v>23</v>
+      </c>
+      <c r="M52" t="s">
+        <v>40</v>
+      </c>
+      <c r="N52" s="1">
+        <v>45901</v>
+      </c>
+      <c r="O52" s="1">
+        <v>46265</v>
+      </c>
+      <c r="P52" s="1">
+        <v>45990</v>
+      </c>
+      <c r="R52" s="1">
+        <v>45661</v>
+      </c>
+      <c r="S52" s="1">
+        <v>48992</v>
+      </c>
+      <c r="T52" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="53" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53">
+        <v>6122</v>
+      </c>
+      <c r="C53" t="s">
+        <v>165</v>
+      </c>
+      <c r="D53" t="s">
+        <v>166</v>
+      </c>
+      <c r="E53">
+        <v>6</v>
+      </c>
+      <c r="F53" t="s">
+        <v>37</v>
+      </c>
+      <c r="G53" t="s">
+        <v>38</v>
+      </c>
+      <c r="H53" t="s">
+        <v>154</v>
+      </c>
+      <c r="I53">
+        <v>2800</v>
+      </c>
+      <c r="J53">
+        <v>0</v>
+      </c>
+      <c r="K53">
+        <v>0</v>
+      </c>
+      <c r="L53" t="s">
+        <v>23</v>
+      </c>
+      <c r="M53" t="s">
+        <v>40</v>
+      </c>
+      <c r="N53" s="1">
+        <v>45645</v>
+      </c>
+      <c r="O53" s="1">
+        <v>46009</v>
+      </c>
+      <c r="P53" s="1">
+        <v>45734</v>
+      </c>
+      <c r="R53" s="1">
+        <v>46361</v>
+      </c>
+      <c r="T53" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="54" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54">
+        <v>6120</v>
+      </c>
+      <c r="C54" t="s">
+        <v>167</v>
+      </c>
+      <c r="D54" t="s">
+        <v>168</v>
+      </c>
+      <c r="E54">
+        <v>6</v>
+      </c>
+      <c r="F54" t="s">
+        <v>37</v>
+      </c>
+      <c r="G54" t="s">
+        <v>38</v>
+      </c>
+      <c r="H54" t="s">
+        <v>154</v>
+      </c>
+      <c r="I54">
+        <v>2800</v>
+      </c>
+      <c r="J54">
+        <v>0</v>
+      </c>
+      <c r="K54">
+        <v>0</v>
+      </c>
+      <c r="L54" t="s">
+        <v>23</v>
+      </c>
+      <c r="M54" t="s">
+        <v>40</v>
+      </c>
+      <c r="N54" s="1">
+        <v>45645</v>
+      </c>
+      <c r="O54" s="1">
+        <v>46009</v>
+      </c>
+      <c r="P54" s="1">
+        <v>45734</v>
+      </c>
+      <c r="R54" s="1">
+        <v>45698</v>
+      </c>
+      <c r="T54" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55">
+        <v>6092</v>
+      </c>
+      <c r="C55" t="s">
+        <v>169</v>
+      </c>
+      <c r="D55" t="s">
+        <v>170</v>
+      </c>
+      <c r="E55">
+        <v>6</v>
+      </c>
+      <c r="F55" t="s">
+        <v>66</v>
+      </c>
+      <c r="G55" t="s">
+        <v>164</v>
+      </c>
+      <c r="H55" t="s">
+        <v>154</v>
+      </c>
+      <c r="I55">
+        <v>2800</v>
+      </c>
+      <c r="J55">
+        <v>0</v>
+      </c>
+      <c r="K55">
+        <v>0</v>
+      </c>
+      <c r="L55" t="s">
+        <v>23</v>
+      </c>
+      <c r="M55" t="s">
+        <v>40</v>
+      </c>
+      <c r="N55" s="1">
+        <v>45637</v>
+      </c>
+      <c r="O55" s="1">
+        <v>46001</v>
+      </c>
+      <c r="P55" s="1">
+        <v>45726</v>
+      </c>
+      <c r="R55" s="1">
+        <v>44933</v>
+      </c>
+      <c r="T55" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="56" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56">
+        <v>6086</v>
+      </c>
+      <c r="C56" t="s">
+        <v>171</v>
+      </c>
+      <c r="D56" t="s">
+        <v>172</v>
+      </c>
+      <c r="E56">
+        <v>6</v>
+      </c>
+      <c r="F56" t="s">
+        <v>37</v>
+      </c>
+      <c r="G56" t="s">
+        <v>173</v>
+      </c>
+      <c r="H56" t="s">
+        <v>174</v>
+      </c>
+      <c r="I56">
+        <v>2800</v>
+      </c>
+      <c r="J56">
+        <v>0</v>
+      </c>
+      <c r="K56">
+        <v>0</v>
+      </c>
+      <c r="L56" t="s">
+        <v>23</v>
+      </c>
+      <c r="M56" t="s">
+        <v>40</v>
+      </c>
+      <c r="N56" s="1">
+        <v>45641</v>
+      </c>
+      <c r="O56" s="1">
+        <v>46005</v>
+      </c>
+      <c r="P56" s="1">
+        <v>45730</v>
+      </c>
+      <c r="R56" s="1">
+        <v>46794</v>
+      </c>
+      <c r="S56" s="1">
+        <v>49191</v>
+      </c>
+      <c r="T56" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="57" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57">
+        <v>6085</v>
+      </c>
+      <c r="C57" t="s">
+        <v>175</v>
+      </c>
+      <c r="D57" t="s">
+        <v>176</v>
+      </c>
+      <c r="E57">
+        <v>6</v>
+      </c>
+      <c r="F57" t="s">
+        <v>37</v>
+      </c>
+      <c r="G57" t="s">
+        <v>173</v>
+      </c>
+      <c r="H57" t="s">
+        <v>174</v>
+      </c>
+      <c r="I57">
+        <v>2800</v>
+      </c>
+      <c r="J57">
+        <v>0</v>
+      </c>
+      <c r="K57">
+        <v>0</v>
+      </c>
+      <c r="L57" t="s">
+        <v>23</v>
+      </c>
+      <c r="M57" t="s">
+        <v>40</v>
+      </c>
+      <c r="N57" s="1">
+        <v>45641</v>
+      </c>
+      <c r="O57" s="1">
+        <v>46005</v>
+      </c>
+      <c r="P57" s="1">
+        <v>45730</v>
+      </c>
+      <c r="R57" s="1">
+        <v>46008</v>
+      </c>
+      <c r="S57" s="1">
+        <v>48099</v>
+      </c>
+      <c r="T57" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="58" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58">
+        <v>5995</v>
+      </c>
+      <c r="C58" t="s">
+        <v>177</v>
+      </c>
+      <c r="D58" t="s">
+        <v>178</v>
+      </c>
+      <c r="E58">
+        <v>6</v>
+      </c>
+      <c r="F58" t="s">
+        <v>32</v>
+      </c>
+      <c r="G58" t="s">
+        <v>43</v>
+      </c>
+      <c r="H58" t="s">
+        <v>154</v>
+      </c>
+      <c r="I58">
+        <v>2800</v>
+      </c>
+      <c r="J58">
+        <v>0</v>
+      </c>
+      <c r="K58">
+        <v>0</v>
+      </c>
+      <c r="L58" t="s">
+        <v>23</v>
+      </c>
+      <c r="M58" t="s">
+        <v>40</v>
+      </c>
+      <c r="N58" s="1">
+        <v>45583</v>
+      </c>
+      <c r="O58" s="1">
+        <v>45947</v>
+      </c>
+      <c r="P58" s="1">
+        <v>45672</v>
+      </c>
+      <c r="R58" s="1">
+        <v>45652</v>
+      </c>
+      <c r="T58" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="59" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59">
+        <v>5993</v>
+      </c>
+      <c r="C59" t="s">
+        <v>179</v>
+      </c>
+      <c r="D59" t="s">
+        <v>180</v>
+      </c>
+      <c r="E59">
+        <v>6</v>
+      </c>
+      <c r="F59" t="s">
+        <v>32</v>
+      </c>
+      <c r="G59" t="s">
+        <v>43</v>
+      </c>
+      <c r="H59" t="s">
+        <v>154</v>
+      </c>
+      <c r="I59">
+        <v>2800</v>
+      </c>
+      <c r="J59">
+        <v>0</v>
+      </c>
+      <c r="K59">
+        <v>0</v>
+      </c>
+      <c r="L59" t="s">
+        <v>23</v>
+      </c>
+      <c r="M59" t="s">
+        <v>40</v>
+      </c>
+      <c r="N59" s="1">
+        <v>45569</v>
+      </c>
+      <c r="O59" s="1">
+        <v>45933</v>
+      </c>
+      <c r="P59" s="1">
+        <v>45658</v>
+      </c>
+      <c r="R59" s="1">
+        <v>45652</v>
+      </c>
+      <c r="S59" s="1">
+        <v>48876</v>
+      </c>
+      <c r="T59" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="60" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60">
+        <v>5961</v>
+      </c>
+      <c r="C60" t="s">
+        <v>181</v>
+      </c>
+      <c r="D60" t="s">
+        <v>182</v>
+      </c>
+      <c r="E60">
+        <v>6</v>
+      </c>
+      <c r="F60" t="s">
+        <v>37</v>
+      </c>
+      <c r="G60" t="s">
+        <v>38</v>
+      </c>
+      <c r="H60" t="s">
+        <v>154</v>
+      </c>
+      <c r="I60">
+        <v>2800</v>
+      </c>
+      <c r="J60">
+        <v>0</v>
+      </c>
+      <c r="K60">
+        <v>0</v>
+      </c>
+      <c r="L60" t="s">
+        <v>23</v>
+      </c>
+      <c r="M60" t="s">
+        <v>40</v>
+      </c>
+      <c r="N60" s="1">
+        <v>45536</v>
+      </c>
+      <c r="O60" s="1">
+        <v>45900</v>
+      </c>
+      <c r="P60" s="1">
+        <v>45625</v>
+      </c>
+      <c r="R60" s="1">
+        <v>45783</v>
+      </c>
+      <c r="T60" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61">
+        <v>5830</v>
+      </c>
+      <c r="C61" t="s">
+        <v>183</v>
+      </c>
+      <c r="D61" t="s">
+        <v>184</v>
+      </c>
+      <c r="E61">
+        <v>6</v>
+      </c>
+      <c r="F61" t="s">
+        <v>37</v>
+      </c>
+      <c r="G61" t="s">
+        <v>173</v>
+      </c>
+      <c r="H61" t="s">
+        <v>174</v>
+      </c>
+      <c r="I61">
+        <v>2800</v>
+      </c>
+      <c r="J61">
+        <v>0</v>
+      </c>
+      <c r="K61">
+        <v>0</v>
+      </c>
+      <c r="L61" t="s">
+        <v>23</v>
+      </c>
+      <c r="M61" t="s">
+        <v>40</v>
+      </c>
+      <c r="N61" s="1">
+        <v>45515</v>
+      </c>
+      <c r="O61" s="1">
+        <v>45879</v>
+      </c>
+      <c r="P61" s="1">
+        <v>45604</v>
+      </c>
+      <c r="Q61" s="1">
+        <v>46323</v>
+      </c>
+      <c r="R61" s="1">
+        <v>45979</v>
+      </c>
+      <c r="T61" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="62" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62">
+        <v>5773</v>
+      </c>
+      <c r="C62" t="s">
+        <v>185</v>
+      </c>
+      <c r="D62" t="s">
+        <v>186</v>
+      </c>
+      <c r="E62">
+        <v>6</v>
+      </c>
+      <c r="F62" t="s">
+        <v>37</v>
+      </c>
+      <c r="G62" t="s">
+        <v>38</v>
+      </c>
+      <c r="H62" t="s">
+        <v>154</v>
+      </c>
+      <c r="I62">
+        <v>2800</v>
+      </c>
+      <c r="J62">
+        <v>0</v>
+      </c>
+      <c r="K62">
+        <v>0</v>
+      </c>
+      <c r="L62" t="s">
+        <v>23</v>
+      </c>
+      <c r="M62" t="s">
+        <v>40</v>
+      </c>
+      <c r="N62" s="1">
+        <v>45485</v>
+      </c>
+      <c r="O62" s="1">
+        <v>45849</v>
+      </c>
+      <c r="P62" s="1">
+        <v>45574</v>
+      </c>
+      <c r="R62" s="1">
+        <v>45661</v>
+      </c>
+      <c r="T62" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="63" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63">
+        <v>6461</v>
+      </c>
+      <c r="C63" t="s">
+        <v>187</v>
+      </c>
+      <c r="D63" t="s">
+        <v>188</v>
+      </c>
+      <c r="E63">
+        <v>6</v>
+      </c>
+      <c r="F63" t="s">
+        <v>32</v>
+      </c>
+      <c r="G63" t="s">
+        <v>43</v>
+      </c>
+      <c r="H63" t="s">
+        <v>154</v>
+      </c>
+      <c r="I63">
+        <v>2800</v>
+      </c>
+      <c r="J63">
+        <v>0</v>
+      </c>
+      <c r="K63">
+        <v>0</v>
+      </c>
+      <c r="L63" t="s">
+        <v>23</v>
+      </c>
+      <c r="M63" t="s">
+        <v>40</v>
+      </c>
+      <c r="N63" s="1">
+        <v>45854</v>
+      </c>
+      <c r="O63" s="1">
+        <v>46189</v>
+      </c>
+      <c r="P63" s="1">
+        <v>45943</v>
+      </c>
+      <c r="R63" s="1">
+        <v>45858</v>
+      </c>
+      <c r="T63" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64">
+        <v>5484</v>
+      </c>
+      <c r="C64" t="s">
+        <v>189</v>
+      </c>
+      <c r="D64" t="s">
+        <v>190</v>
+      </c>
+      <c r="E64">
+        <v>6</v>
+      </c>
+      <c r="F64" t="s">
+        <v>37</v>
+      </c>
+      <c r="G64" t="s">
+        <v>173</v>
+      </c>
+      <c r="H64" t="s">
+        <v>174</v>
+      </c>
+      <c r="I64">
+        <v>2800</v>
+      </c>
+      <c r="J64">
+        <v>0</v>
+      </c>
+      <c r="K64">
+        <v>0</v>
+      </c>
+      <c r="L64" t="s">
+        <v>23</v>
+      </c>
+      <c r="M64" t="s">
+        <v>40</v>
+      </c>
+      <c r="N64" s="1">
+        <v>45216</v>
+      </c>
+      <c r="O64" s="1">
+        <v>45581</v>
+      </c>
+      <c r="P64" s="1">
+        <v>45305</v>
+      </c>
+      <c r="R64" s="1">
+        <v>45117</v>
+      </c>
+      <c r="T64" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="65" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65">
+        <v>6589</v>
+      </c>
+      <c r="C65" t="s">
+        <v>191</v>
+      </c>
+      <c r="D65" t="s">
+        <v>192</v>
+      </c>
+      <c r="E65">
+        <v>6</v>
+      </c>
+      <c r="F65" t="s">
+        <v>37</v>
+      </c>
+      <c r="G65" t="s">
+        <v>38</v>
+      </c>
+      <c r="H65" t="s">
+        <v>154</v>
+      </c>
+      <c r="I65">
+        <v>2800</v>
+      </c>
+      <c r="J65">
+        <v>0</v>
+      </c>
+      <c r="K65">
+        <v>0</v>
+      </c>
+      <c r="L65" t="s">
+        <v>23</v>
+      </c>
+      <c r="M65" t="s">
+        <v>40</v>
+      </c>
+      <c r="N65" s="1">
+        <v>45874</v>
+      </c>
+      <c r="O65" s="1">
+        <v>46238</v>
+      </c>
+      <c r="P65" s="1">
+        <v>45963</v>
+      </c>
+      <c r="S65" s="1">
+        <v>48500</v>
+      </c>
+      <c r="T65" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="66" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66">
+        <v>5128</v>
+      </c>
+      <c r="C66" t="s">
+        <v>194</v>
+      </c>
+      <c r="D66" t="s">
+        <v>195</v>
+      </c>
+      <c r="E66">
+        <v>6</v>
+      </c>
+      <c r="F66" t="s">
+        <v>66</v>
+      </c>
+      <c r="G66" t="s">
+        <v>164</v>
+      </c>
+      <c r="H66" t="s">
+        <v>154</v>
+      </c>
+      <c r="I66">
+        <v>2800</v>
+      </c>
+      <c r="J66">
+        <v>0</v>
+      </c>
+      <c r="K66">
+        <v>0</v>
+      </c>
+      <c r="L66" t="s">
+        <v>23</v>
+      </c>
+      <c r="M66" t="s">
+        <v>40</v>
+      </c>
+      <c r="N66" s="1">
+        <v>44808</v>
+      </c>
+      <c r="O66" s="1">
+        <v>45172</v>
+      </c>
+      <c r="P66" s="1">
+        <v>44898</v>
+      </c>
+      <c r="R66" s="1">
+        <v>46319</v>
+      </c>
+      <c r="T66" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="67" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67">
+        <v>6675</v>
+      </c>
+      <c r="C67" t="s">
+        <v>196</v>
+      </c>
+      <c r="D67" t="s">
+        <v>197</v>
+      </c>
+      <c r="E67">
+        <v>6</v>
+      </c>
+      <c r="F67" t="s">
+        <v>32</v>
+      </c>
+      <c r="G67" t="s">
+        <v>43</v>
+      </c>
+      <c r="H67" t="s">
+        <v>154</v>
+      </c>
+      <c r="I67">
+        <v>2800</v>
+      </c>
+      <c r="J67">
+        <v>0</v>
+      </c>
+      <c r="K67">
+        <v>0</v>
+      </c>
+      <c r="L67" t="s">
+        <v>23</v>
+      </c>
+      <c r="M67" t="s">
+        <v>40</v>
+      </c>
+      <c r="N67" s="1">
+        <v>46204</v>
+      </c>
+      <c r="P67" s="1">
+        <v>46203</v>
+      </c>
+      <c r="T67" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="68" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68">
+        <v>2650</v>
+      </c>
+      <c r="C68" t="s">
+        <v>199</v>
+      </c>
+      <c r="D68" t="s">
+        <v>200</v>
+      </c>
+      <c r="E68">
+        <v>6</v>
+      </c>
+      <c r="F68" t="s">
+        <v>46</v>
+      </c>
+      <c r="G68" t="s">
+        <v>153</v>
+      </c>
+      <c r="H68" t="s">
+        <v>154</v>
+      </c>
+      <c r="I68">
+        <v>2800</v>
+      </c>
+      <c r="J68">
+        <v>0</v>
+      </c>
+      <c r="K68">
+        <v>0</v>
+      </c>
+      <c r="L68" t="s">
+        <v>23</v>
+      </c>
+      <c r="M68" t="s">
+        <v>40</v>
+      </c>
+      <c r="N68" s="1">
+        <v>46244</v>
+      </c>
+      <c r="P68" s="1">
+        <v>46243</v>
+      </c>
+      <c r="R68" s="1">
+        <v>46216</v>
+      </c>
+      <c r="T68" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="69" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69">
+        <v>2649</v>
+      </c>
+      <c r="C69" t="s">
+        <v>201</v>
+      </c>
+      <c r="D69" t="s">
+        <v>202</v>
+      </c>
+      <c r="E69">
+        <v>6</v>
+      </c>
+      <c r="F69" t="s">
+        <v>46</v>
+      </c>
+      <c r="G69" t="s">
+        <v>153</v>
+      </c>
+      <c r="H69" t="s">
+        <v>154</v>
+      </c>
+      <c r="I69">
+        <v>2800</v>
+      </c>
+      <c r="J69">
+        <v>0</v>
+      </c>
+      <c r="K69">
+        <v>0</v>
+      </c>
+      <c r="L69" t="s">
+        <v>23</v>
+      </c>
+      <c r="M69" t="s">
+        <v>40</v>
+      </c>
+      <c r="N69" s="1">
+        <v>46244</v>
+      </c>
+      <c r="P69" s="1">
+        <v>46243</v>
+      </c>
+      <c r="R69" s="1">
+        <v>45729</v>
+      </c>
+      <c r="T69" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="70" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70">
+        <v>6166</v>
+      </c>
+      <c r="C70" t="s">
+        <v>203</v>
+      </c>
+      <c r="D70" t="s">
+        <v>204</v>
+      </c>
+      <c r="E70">
+        <v>6</v>
+      </c>
+      <c r="F70" t="s">
+        <v>32</v>
+      </c>
+      <c r="G70" t="s">
+        <v>43</v>
+      </c>
+      <c r="H70" t="s">
+        <v>154</v>
+      </c>
+      <c r="I70">
+        <v>2800</v>
+      </c>
+      <c r="J70">
+        <v>0</v>
+      </c>
+      <c r="K70">
+        <v>0</v>
+      </c>
+      <c r="L70" t="s">
+        <v>23</v>
+      </c>
+      <c r="M70" t="s">
+        <v>40</v>
+      </c>
+      <c r="N70" s="1">
+        <v>45658</v>
+      </c>
+      <c r="O70" s="1">
+        <v>46022</v>
+      </c>
+      <c r="P70" s="1">
+        <v>45747</v>
+      </c>
+      <c r="R70" s="1">
+        <v>45661</v>
+      </c>
+      <c r="T70" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71">
+        <v>7287</v>
+      </c>
+      <c r="C71" t="s">
+        <v>205</v>
+      </c>
+      <c r="D71" t="s">
+        <v>206</v>
+      </c>
+      <c r="E71">
+        <v>6</v>
+      </c>
+      <c r="F71" t="s">
+        <v>46</v>
+      </c>
+      <c r="G71" t="s">
+        <v>153</v>
+      </c>
+      <c r="H71" t="s">
+        <v>154</v>
+      </c>
+      <c r="I71">
+        <v>2800</v>
+      </c>
+      <c r="J71">
+        <v>0</v>
+      </c>
+      <c r="K71">
+        <v>0</v>
+      </c>
+      <c r="L71" t="s">
+        <v>23</v>
+      </c>
+      <c r="M71" t="s">
+        <v>40</v>
+      </c>
+      <c r="N71" s="1">
+        <v>46223</v>
+      </c>
+      <c r="P71" s="1">
+        <v>46222</v>
+      </c>
+      <c r="T71" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="72" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72">
+        <v>7288</v>
+      </c>
+      <c r="C72" t="s">
+        <v>207</v>
+      </c>
+      <c r="D72" t="s">
+        <v>208</v>
+      </c>
+      <c r="E72">
+        <v>6</v>
+      </c>
+      <c r="F72" t="s">
+        <v>46</v>
+      </c>
+      <c r="G72" t="s">
+        <v>153</v>
+      </c>
+      <c r="H72" t="s">
+        <v>154</v>
+      </c>
+      <c r="I72">
+        <v>2800</v>
+      </c>
+      <c r="J72">
+        <v>0</v>
+      </c>
+      <c r="K72">
+        <v>0</v>
+      </c>
+      <c r="L72" t="s">
+        <v>23</v>
+      </c>
+      <c r="M72" t="s">
+        <v>40</v>
+      </c>
+      <c r="N72" s="1">
+        <v>46219</v>
+      </c>
+      <c r="P72" s="1">
+        <v>46218</v>
+      </c>
+      <c r="T72" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="73" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73">
+        <v>7289</v>
+      </c>
+      <c r="C73" t="s">
+        <v>209</v>
+      </c>
+      <c r="D73" t="s">
+        <v>210</v>
+      </c>
+      <c r="E73">
+        <v>6</v>
+      </c>
+      <c r="F73" t="s">
+        <v>46</v>
+      </c>
+      <c r="G73" t="s">
+        <v>153</v>
+      </c>
+      <c r="H73" t="s">
+        <v>154</v>
+      </c>
+      <c r="I73">
+        <v>2800</v>
+      </c>
+      <c r="J73">
+        <v>0</v>
+      </c>
+      <c r="K73">
+        <v>0</v>
+      </c>
+      <c r="L73" t="s">
+        <v>23</v>
+      </c>
+      <c r="M73" t="s">
+        <v>40</v>
+      </c>
+      <c r="N73" s="1">
+        <v>46219</v>
+      </c>
+      <c r="P73" s="1">
+        <v>46218</v>
+      </c>
+      <c r="T73" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="74" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74">
+        <v>7291</v>
+      </c>
+      <c r="C74" t="s">
+        <v>211</v>
+      </c>
+      <c r="D74" t="s">
+        <v>212</v>
+      </c>
+      <c r="E74">
+        <v>6</v>
+      </c>
+      <c r="F74" t="s">
+        <v>46</v>
+      </c>
+      <c r="G74" t="s">
+        <v>153</v>
+      </c>
+      <c r="H74" t="s">
+        <v>154</v>
+      </c>
+      <c r="I74">
+        <v>2800</v>
+      </c>
+      <c r="J74">
+        <v>0</v>
+      </c>
+      <c r="K74">
+        <v>0</v>
+      </c>
+      <c r="L74" t="s">
+        <v>23</v>
+      </c>
+      <c r="M74" t="s">
+        <v>40</v>
+      </c>
+      <c r="N74" s="1">
+        <v>46219</v>
+      </c>
+      <c r="P74" s="1">
+        <v>46218</v>
+      </c>
+      <c r="T74" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="75" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75">
+        <v>7292</v>
+      </c>
+      <c r="C75" t="s">
+        <v>213</v>
+      </c>
+      <c r="D75" t="s">
+        <v>214</v>
+      </c>
+      <c r="E75">
+        <v>6</v>
+      </c>
+      <c r="F75" t="s">
+        <v>46</v>
+      </c>
+      <c r="G75" t="s">
+        <v>153</v>
+      </c>
+      <c r="H75" t="s">
+        <v>154</v>
+      </c>
+      <c r="I75">
+        <v>2800</v>
+      </c>
+      <c r="J75">
+        <v>0</v>
+      </c>
+      <c r="K75">
+        <v>0</v>
+      </c>
+      <c r="L75" t="s">
+        <v>23</v>
+      </c>
+      <c r="M75" t="s">
+        <v>40</v>
+      </c>
+      <c r="N75" s="1">
+        <v>46219</v>
+      </c>
+      <c r="P75" s="1">
+        <v>46218</v>
+      </c>
+      <c r="T75" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="76" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76">
+        <v>7293</v>
+      </c>
+      <c r="C76" t="s">
+        <v>215</v>
+      </c>
+      <c r="D76" t="s">
+        <v>216</v>
+      </c>
+      <c r="E76">
+        <v>6</v>
+      </c>
+      <c r="F76" t="s">
+        <v>46</v>
+      </c>
+      <c r="G76" t="s">
+        <v>153</v>
+      </c>
+      <c r="H76" t="s">
+        <v>154</v>
+      </c>
+      <c r="I76">
+        <v>2800</v>
+      </c>
+      <c r="J76">
+        <v>0</v>
+      </c>
+      <c r="K76">
+        <v>0</v>
+      </c>
+      <c r="L76" t="s">
+        <v>23</v>
+      </c>
+      <c r="M76" t="s">
+        <v>40</v>
+      </c>
+      <c r="N76" s="1">
+        <v>46219</v>
+      </c>
+      <c r="P76" s="1">
+        <v>46218</v>
+      </c>
+      <c r="T76" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="77" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77">
+        <v>7294</v>
+      </c>
+      <c r="C77" t="s">
+        <v>217</v>
+      </c>
+      <c r="D77" t="s">
+        <v>218</v>
+      </c>
+      <c r="E77">
+        <v>6</v>
+      </c>
+      <c r="F77" t="s">
+        <v>37</v>
+      </c>
+      <c r="G77" t="s">
+        <v>38</v>
+      </c>
+      <c r="H77" t="s">
+        <v>154</v>
+      </c>
+      <c r="I77">
+        <v>2800</v>
+      </c>
+      <c r="J77">
+        <v>0</v>
+      </c>
+      <c r="K77">
+        <v>0</v>
+      </c>
+      <c r="L77" t="s">
+        <v>23</v>
+      </c>
+      <c r="M77" t="s">
+        <v>40</v>
+      </c>
+      <c r="N77" s="1">
+        <v>46219</v>
+      </c>
+      <c r="P77" s="1">
+        <v>46218</v>
+      </c>
+      <c r="T77" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="78" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78">
+        <v>7295</v>
+      </c>
+      <c r="C78" t="s">
+        <v>219</v>
+      </c>
+      <c r="D78" t="s">
+        <v>220</v>
+      </c>
+      <c r="E78">
+        <v>6</v>
+      </c>
+      <c r="F78" t="s">
+        <v>46</v>
+      </c>
+      <c r="G78" t="s">
+        <v>153</v>
+      </c>
+      <c r="H78" t="s">
+        <v>154</v>
+      </c>
+      <c r="I78">
+        <v>2800</v>
+      </c>
+      <c r="J78">
+        <v>0</v>
+      </c>
+      <c r="K78">
+        <v>0</v>
+      </c>
+      <c r="L78" t="s">
+        <v>23</v>
+      </c>
+      <c r="M78" t="s">
+        <v>40</v>
+      </c>
+      <c r="N78" s="1">
+        <v>46219</v>
+      </c>
+      <c r="P78" s="1">
+        <v>46218</v>
+      </c>
+      <c r="T78" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="79" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79">
+        <v>7300</v>
+      </c>
+      <c r="C79" t="s">
+        <v>221</v>
+      </c>
+      <c r="D79" t="s">
+        <v>222</v>
+      </c>
+      <c r="E79">
+        <v>6</v>
+      </c>
+      <c r="F79" t="s">
+        <v>46</v>
+      </c>
+      <c r="G79" t="s">
+        <v>223</v>
+      </c>
+      <c r="H79" t="s">
+        <v>174</v>
+      </c>
+      <c r="I79">
+        <v>2800</v>
+      </c>
+      <c r="J79">
+        <v>0</v>
+      </c>
+      <c r="K79">
+        <v>0</v>
+      </c>
+      <c r="L79" t="s">
+        <v>23</v>
+      </c>
+      <c r="M79" t="s">
+        <v>40</v>
+      </c>
+      <c r="N79" s="1">
+        <v>46218</v>
+      </c>
+      <c r="O79" s="1">
+        <v>46582</v>
+      </c>
+      <c r="P79" s="1">
+        <v>46307</v>
+      </c>
+      <c r="T79" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="80" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80">
+        <v>7301</v>
+      </c>
+      <c r="C80" t="s">
+        <v>225</v>
+      </c>
+      <c r="D80" t="s">
+        <v>226</v>
+      </c>
+      <c r="E80">
+        <v>6</v>
+      </c>
+      <c r="F80" t="s">
+        <v>46</v>
+      </c>
+      <c r="G80" t="s">
+        <v>223</v>
+      </c>
+      <c r="H80" t="s">
+        <v>174</v>
+      </c>
+      <c r="I80">
+        <v>2800</v>
+      </c>
+      <c r="J80">
+        <v>0</v>
+      </c>
+      <c r="K80">
+        <v>0</v>
+      </c>
+      <c r="L80" t="s">
+        <v>23</v>
+      </c>
+      <c r="M80" t="s">
+        <v>40</v>
+      </c>
+      <c r="N80" s="1">
+        <v>46218</v>
+      </c>
+      <c r="P80" s="1">
+        <v>46217</v>
+      </c>
+      <c r="T80" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="81" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81">
+        <v>7302</v>
+      </c>
+      <c r="C81" t="s">
+        <v>227</v>
+      </c>
+      <c r="D81" t="s">
+        <v>228</v>
+      </c>
+      <c r="E81">
+        <v>6</v>
+      </c>
+      <c r="F81" t="s">
+        <v>46</v>
+      </c>
+      <c r="G81" t="s">
+        <v>223</v>
+      </c>
+      <c r="H81" t="s">
+        <v>174</v>
+      </c>
+      <c r="I81">
+        <v>2800</v>
+      </c>
+      <c r="J81">
+        <v>0</v>
+      </c>
+      <c r="K81">
+        <v>0</v>
+      </c>
+      <c r="L81" t="s">
+        <v>23</v>
+      </c>
+      <c r="M81" t="s">
+        <v>40</v>
+      </c>
+      <c r="N81" s="1">
+        <v>46218</v>
+      </c>
+      <c r="P81" s="1">
+        <v>46217</v>
+      </c>
+      <c r="T81" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="82" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82">
+        <v>6233</v>
+      </c>
+      <c r="C82" t="s">
+        <v>229</v>
+      </c>
+      <c r="D82" t="s">
+        <v>230</v>
+      </c>
+      <c r="E82">
+        <v>6</v>
+      </c>
+      <c r="F82" t="s">
+        <v>66</v>
+      </c>
+      <c r="G82" t="s">
+        <v>164</v>
+      </c>
+      <c r="H82" t="s">
+        <v>154</v>
+      </c>
+      <c r="I82">
+        <v>2800</v>
+      </c>
+      <c r="J82">
+        <v>0</v>
+      </c>
+      <c r="K82">
+        <v>0</v>
+      </c>
+      <c r="L82" t="s">
+        <v>23</v>
+      </c>
+      <c r="M82" t="s">
+        <v>40</v>
+      </c>
+      <c r="N82" s="1">
+        <v>45717</v>
+      </c>
+      <c r="O82" s="1">
+        <v>46081</v>
+      </c>
+      <c r="P82" s="1">
+        <v>45806</v>
+      </c>
+      <c r="R82" s="1">
+        <v>45719</v>
+      </c>
+      <c r="T82" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="83" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83">
+        <v>6234</v>
+      </c>
+      <c r="C83" t="s">
+        <v>231</v>
+      </c>
+      <c r="D83" t="s">
+        <v>232</v>
+      </c>
+      <c r="E83">
+        <v>6</v>
+      </c>
+      <c r="F83" t="s">
+        <v>66</v>
+      </c>
+      <c r="G83" t="s">
+        <v>164</v>
+      </c>
+      <c r="H83" t="s">
+        <v>154</v>
+      </c>
+      <c r="I83">
+        <v>2800</v>
+      </c>
+      <c r="J83">
+        <v>0</v>
+      </c>
+      <c r="K83">
+        <v>0</v>
+      </c>
+      <c r="L83" t="s">
+        <v>23</v>
+      </c>
+      <c r="M83" t="s">
+        <v>40</v>
+      </c>
+      <c r="N83" s="1">
+        <v>45717</v>
+      </c>
+      <c r="O83" s="1">
+        <v>46081</v>
+      </c>
+      <c r="P83" s="1">
+        <v>45806</v>
+      </c>
+      <c r="R83" s="1">
+        <v>45746</v>
+      </c>
+      <c r="T83" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="84" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84">
+        <v>6235</v>
+      </c>
+      <c r="C84" t="s">
+        <v>233</v>
+      </c>
+      <c r="D84" t="s">
+        <v>234</v>
+      </c>
+      <c r="E84">
+        <v>6</v>
+      </c>
+      <c r="F84" t="s">
+        <v>66</v>
+      </c>
+      <c r="G84" t="s">
+        <v>164</v>
+      </c>
+      <c r="H84" t="s">
+        <v>154</v>
+      </c>
+      <c r="I84">
+        <v>2800</v>
+      </c>
+      <c r="J84">
+        <v>0</v>
+      </c>
+      <c r="K84">
+        <v>0</v>
+      </c>
+      <c r="L84" t="s">
+        <v>23</v>
+      </c>
+      <c r="M84" t="s">
+        <v>40</v>
+      </c>
+      <c r="N84" s="1">
+        <v>45717</v>
+      </c>
+      <c r="O84" s="1">
+        <v>46081</v>
+      </c>
+      <c r="P84" s="1">
+        <v>45806</v>
+      </c>
+      <c r="R84" s="1">
+        <v>45718</v>
+      </c>
+      <c r="T84" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="85" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85">
+        <v>6236</v>
+      </c>
+      <c r="C85" t="s">
+        <v>235</v>
+      </c>
+      <c r="D85" t="s">
+        <v>236</v>
+      </c>
+      <c r="E85">
+        <v>6</v>
+      </c>
+      <c r="F85" t="s">
+        <v>66</v>
+      </c>
+      <c r="G85" t="s">
+        <v>164</v>
+      </c>
+      <c r="H85" t="s">
+        <v>154</v>
+      </c>
+      <c r="I85">
+        <v>2800</v>
+      </c>
+      <c r="J85">
+        <v>0</v>
+      </c>
+      <c r="K85">
+        <v>0</v>
+      </c>
+      <c r="L85" t="s">
+        <v>23</v>
+      </c>
+      <c r="M85" t="s">
+        <v>40</v>
+      </c>
+      <c r="N85" s="1">
+        <v>45717</v>
+      </c>
+      <c r="O85" s="1">
+        <v>46081</v>
+      </c>
+      <c r="P85" s="1">
+        <v>45806</v>
+      </c>
+      <c r="R85" s="1">
+        <v>45440</v>
+      </c>
+      <c r="T85" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="86" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86">
+        <v>6237</v>
+      </c>
+      <c r="C86" t="s">
+        <v>237</v>
+      </c>
+      <c r="D86" t="s">
+        <v>238</v>
+      </c>
+      <c r="E86">
+        <v>6</v>
+      </c>
+      <c r="F86" t="s">
+        <v>66</v>
+      </c>
+      <c r="G86" t="s">
+        <v>164</v>
+      </c>
+      <c r="H86" t="s">
+        <v>154</v>
+      </c>
+      <c r="I86">
+        <v>2800</v>
+      </c>
+      <c r="J86">
+        <v>0</v>
+      </c>
+      <c r="K86">
+        <v>0</v>
+      </c>
+      <c r="L86" t="s">
+        <v>23</v>
+      </c>
+      <c r="M86" t="s">
+        <v>40</v>
+      </c>
+      <c r="N86" s="1">
+        <v>45717</v>
+      </c>
+      <c r="O86" s="1">
+        <v>46081</v>
+      </c>
+      <c r="P86" s="1">
+        <v>45806</v>
+      </c>
+      <c r="R86" s="1">
+        <v>46089</v>
+      </c>
+      <c r="T86" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="87" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87">
+        <v>6450</v>
+      </c>
+      <c r="C87" t="s">
+        <v>239</v>
+      </c>
+      <c r="D87" t="s">
+        <v>240</v>
+      </c>
+      <c r="E87">
+        <v>6</v>
+      </c>
+      <c r="F87" t="s">
+        <v>66</v>
+      </c>
+      <c r="G87" t="s">
+        <v>164</v>
+      </c>
+      <c r="H87" t="s">
+        <v>154</v>
+      </c>
+      <c r="I87">
+        <v>2800</v>
+      </c>
+      <c r="J87">
+        <v>0</v>
+      </c>
+      <c r="K87">
+        <v>0</v>
+      </c>
+      <c r="L87" t="s">
+        <v>23</v>
+      </c>
+      <c r="M87" t="s">
+        <v>40</v>
+      </c>
+      <c r="N87" s="1">
+        <v>45854</v>
+      </c>
+      <c r="O87" s="1">
+        <v>46218</v>
+      </c>
+      <c r="P87" s="1">
+        <v>45943</v>
+      </c>
+      <c r="T87" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="88" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88">
+        <v>6455</v>
+      </c>
+      <c r="C88" t="s">
+        <v>241</v>
+      </c>
+      <c r="D88" t="s">
+        <v>242</v>
+      </c>
+      <c r="E88">
+        <v>6</v>
+      </c>
+      <c r="F88" t="s">
+        <v>66</v>
+      </c>
+      <c r="G88" t="s">
+        <v>164</v>
+      </c>
+      <c r="H88" t="s">
+        <v>154</v>
+      </c>
+      <c r="I88">
+        <v>2800</v>
+      </c>
+      <c r="J88">
+        <v>0</v>
+      </c>
+      <c r="K88">
+        <v>0</v>
+      </c>
+      <c r="L88" t="s">
+        <v>23</v>
+      </c>
+      <c r="M88" t="s">
+        <v>40</v>
+      </c>
+      <c r="N88" s="1">
+        <v>45854</v>
+      </c>
+      <c r="O88" s="1">
+        <v>46218</v>
+      </c>
+      <c r="P88" s="1">
+        <v>45943</v>
+      </c>
+      <c r="T88" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="89" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89">
+        <v>6459</v>
+      </c>
+      <c r="C89" t="s">
+        <v>243</v>
+      </c>
+      <c r="D89" t="s">
+        <v>244</v>
+      </c>
+      <c r="E89">
+        <v>6</v>
+      </c>
+      <c r="F89" t="s">
+        <v>32</v>
+      </c>
+      <c r="G89" t="s">
+        <v>43</v>
+      </c>
+      <c r="H89" t="s">
+        <v>154</v>
+      </c>
+      <c r="I89">
+        <v>2800</v>
+      </c>
+      <c r="J89">
+        <v>0</v>
+      </c>
+      <c r="K89">
+        <v>0</v>
+      </c>
+      <c r="L89" t="s">
+        <v>23</v>
+      </c>
+      <c r="M89" t="s">
+        <v>40</v>
+      </c>
+      <c r="N89" s="1">
+        <v>45854</v>
+      </c>
+      <c r="O89" s="1">
+        <v>46218</v>
+      </c>
+      <c r="P89" s="1">
+        <v>45943</v>
+      </c>
+      <c r="S89" s="1">
+        <v>48602</v>
+      </c>
+      <c r="T89" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="90" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90">
+        <v>6460</v>
+      </c>
+      <c r="C90" t="s">
+        <v>245</v>
+      </c>
+      <c r="D90" t="s">
+        <v>246</v>
+      </c>
+      <c r="E90">
+        <v>6</v>
+      </c>
+      <c r="F90" t="s">
+        <v>32</v>
+      </c>
+      <c r="G90" t="s">
+        <v>43</v>
+      </c>
+      <c r="H90" t="s">
+        <v>154</v>
+      </c>
+      <c r="I90">
+        <v>2800</v>
+      </c>
+      <c r="J90">
+        <v>0</v>
+      </c>
+      <c r="K90">
+        <v>0</v>
+      </c>
+      <c r="L90" t="s">
+        <v>23</v>
+      </c>
+      <c r="M90" t="s">
+        <v>40</v>
+      </c>
+      <c r="N90" s="1">
+        <v>45854</v>
+      </c>
+      <c r="O90" s="1">
+        <v>46218</v>
+      </c>
+      <c r="P90" s="1">
+        <v>45943</v>
+      </c>
+      <c r="T90" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="91" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91">
+        <v>6587</v>
+      </c>
+      <c r="C91" t="s">
+        <v>247</v>
+      </c>
+      <c r="D91" t="s">
+        <v>248</v>
+      </c>
+      <c r="E91">
+        <v>6</v>
+      </c>
+      <c r="F91" t="s">
+        <v>37</v>
+      </c>
+      <c r="G91" t="s">
+        <v>38</v>
+      </c>
+      <c r="H91" t="s">
+        <v>154</v>
+      </c>
+      <c r="I91">
+        <v>2800</v>
+      </c>
+      <c r="J91">
+        <v>0</v>
+      </c>
+      <c r="K91">
+        <v>0</v>
+      </c>
+      <c r="L91" t="s">
+        <v>23</v>
+      </c>
+      <c r="M91" t="s">
+        <v>40</v>
+      </c>
+      <c r="N91" s="1">
+        <v>45874</v>
+      </c>
+      <c r="O91" s="1">
+        <v>46238</v>
+      </c>
+      <c r="P91" s="1">
+        <v>45963</v>
+      </c>
+      <c r="T91" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="92" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92">
+        <v>6674</v>
+      </c>
+      <c r="C92" t="s">
+        <v>249</v>
+      </c>
+      <c r="D92" t="s">
+        <v>250</v>
+      </c>
+      <c r="E92">
+        <v>5</v>
+      </c>
+      <c r="F92" t="s">
+        <v>37</v>
+      </c>
+      <c r="G92" t="s">
+        <v>38</v>
+      </c>
+      <c r="H92" t="s">
+        <v>251</v>
+      </c>
+      <c r="I92">
+        <v>2800</v>
+      </c>
+      <c r="J92">
+        <v>0</v>
+      </c>
+      <c r="K92">
+        <v>0</v>
+      </c>
+      <c r="L92" t="s">
+        <v>23</v>
+      </c>
+      <c r="M92" t="s">
+        <v>40</v>
+      </c>
+      <c r="N92" s="1">
+        <v>45992</v>
+      </c>
+      <c r="P92" s="1">
+        <v>45991</v>
+      </c>
+      <c r="T92" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="93" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93">
+        <v>7648</v>
+      </c>
+      <c r="C93" t="s">
+        <v>252</v>
+      </c>
+      <c r="D93" t="s">
+        <v>253</v>
+      </c>
+      <c r="E93">
+        <v>6</v>
+      </c>
+      <c r="F93" t="s">
+        <v>46</v>
+      </c>
+      <c r="G93" t="s">
+        <v>153</v>
+      </c>
+      <c r="H93" t="s">
+        <v>154</v>
+      </c>
+      <c r="I93">
+        <v>2800</v>
+      </c>
+      <c r="J93">
+        <v>0</v>
+      </c>
+      <c r="K93">
+        <v>0</v>
+      </c>
+      <c r="L93" t="s">
+        <v>23</v>
+      </c>
+      <c r="M93" t="s">
+        <v>40</v>
+      </c>
+      <c r="N93" s="1">
+        <v>46244</v>
+      </c>
+      <c r="P93" s="1">
+        <v>46243</v>
+      </c>
+      <c r="R93" s="1">
+        <v>46113</v>
+      </c>
+      <c r="T93" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="94" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94">
+        <v>8008</v>
+      </c>
+      <c r="C94" t="s">
+        <v>254</v>
+      </c>
+      <c r="D94" t="s">
+        <v>255</v>
+      </c>
+      <c r="E94">
+        <v>6</v>
+      </c>
+      <c r="F94" t="s">
+        <v>32</v>
+      </c>
+      <c r="G94" t="s">
+        <v>43</v>
+      </c>
+      <c r="H94" t="s">
+        <v>154</v>
+      </c>
+      <c r="I94">
+        <v>2800</v>
+      </c>
+      <c r="J94">
+        <v>0</v>
+      </c>
+      <c r="K94">
+        <v>0</v>
+      </c>
+      <c r="L94" t="s">
+        <v>23</v>
+      </c>
+      <c r="M94" t="s">
+        <v>40</v>
+      </c>
+      <c r="N94" s="1">
+        <v>46305</v>
+      </c>
+      <c r="R94" s="1">
+        <v>46377</v>
+      </c>
+      <c r="T94" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="95" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95">
+        <v>7277</v>
+      </c>
+      <c r="C95" t="s">
+        <v>256</v>
+      </c>
+      <c r="D95" t="s">
+        <v>257</v>
+      </c>
+      <c r="E95">
+        <v>6</v>
+      </c>
+      <c r="F95" t="s">
+        <v>37</v>
+      </c>
+      <c r="G95" t="s">
+        <v>38</v>
+      </c>
+      <c r="H95" t="s">
+        <v>154</v>
+      </c>
+      <c r="I95">
+        <v>2800</v>
+      </c>
+      <c r="J95">
+        <v>0</v>
+      </c>
+      <c r="K95">
+        <v>0</v>
+      </c>
+      <c r="L95" t="s">
+        <v>23</v>
+      </c>
+      <c r="M95" t="s">
+        <v>40</v>
+      </c>
+      <c r="N95" s="1">
+        <v>46143</v>
+      </c>
+      <c r="O95" s="1">
+        <v>46507</v>
+      </c>
+      <c r="P95" s="1">
+        <v>46232</v>
+      </c>
+      <c r="T95" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="96" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96">
+        <v>7278</v>
+      </c>
+      <c r="C96" t="s">
+        <v>258</v>
+      </c>
+      <c r="D96" t="s">
+        <v>259</v>
+      </c>
+      <c r="E96">
+        <v>6</v>
+      </c>
+      <c r="F96" t="s">
+        <v>37</v>
+      </c>
+      <c r="G96" t="s">
+        <v>38</v>
+      </c>
+      <c r="H96" t="s">
+        <v>154</v>
+      </c>
+      <c r="I96">
+        <v>2800</v>
+      </c>
+      <c r="J96">
+        <v>0</v>
+      </c>
+      <c r="K96">
+        <v>0</v>
+      </c>
+      <c r="L96" t="s">
+        <v>23</v>
+      </c>
+      <c r="M96" t="s">
+        <v>40</v>
+      </c>
+      <c r="N96" s="1">
+        <v>46143</v>
+      </c>
+      <c r="O96" s="1">
+        <v>46507</v>
+      </c>
+      <c r="P96" s="1">
+        <v>46232</v>
+      </c>
+      <c r="T96" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="97" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97">
+        <v>7286</v>
+      </c>
+      <c r="C97" t="s">
+        <v>260</v>
+      </c>
+      <c r="D97" t="s">
+        <v>261</v>
+      </c>
+      <c r="E97">
+        <v>6</v>
+      </c>
+      <c r="F97" t="s">
+        <v>32</v>
+      </c>
+      <c r="G97" t="s">
+        <v>43</v>
+      </c>
+      <c r="H97" t="s">
+        <v>154</v>
+      </c>
+      <c r="I97">
+        <v>2800</v>
+      </c>
+      <c r="J97">
+        <v>0</v>
+      </c>
+      <c r="K97">
+        <v>0</v>
+      </c>
+      <c r="L97" t="s">
+        <v>23</v>
+      </c>
+      <c r="M97" t="s">
+        <v>40</v>
+      </c>
+      <c r="N97" s="1">
+        <v>46219</v>
+      </c>
+      <c r="P97" s="1">
+        <v>46218</v>
+      </c>
+      <c r="T97" t="s">
+        <v>155</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>